<commit_message>
feat: implement audit logging for dataset mutations and update documentation
</commit_message>
<xml_diff>
--- a/examples/workbook.xlsx
+++ b/examples/workbook.xlsx
@@ -639,7 +639,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -717,15 +717,24 @@
           <t>Car Part</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>99.00</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="B6" t="n">
+        <v>99</v>
+      </c>
+      <c r="C6" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>foobar</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>99</v>
+      </c>
+      <c r="C7" t="n">
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>